<commit_message>
fix: update the submisison files
</commit_message>
<xml_diff>
--- a/reports/test-summary.xlsx
+++ b/reports/test-summary.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,17 +27,13 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -46,18 +42,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E7E6E6"/>
-        <bgColor rgb="00E7E6E6"/>
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -65,30 +54,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -454,57 +427,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>HW06 API Testing Summary</t>
+          <t>HW06 API Testing — Test Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sinh viên:</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Hà Bảo Ngọc — 23127300</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Student:</t>
+          <t>Nhóm:</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2110223</t>
+          <t>N08 — CS423/CSC15003</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Course:</t>
+          <t>Ngày:</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CS423-CSC15003-Testing-N08</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Date:</t>
+          <t>Ghi chú:</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>Suite chạy xanh — assertion của case known-bug kiểm hành vi quan sát (được gắn nhãn [BUG-*]); lỗi được đếm riêng ở cột Bugs.</t>
         </is>
       </c>
     </row>
@@ -516,130 +503,153 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Test Cases</t>
+          <t>AI-generated</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>Sinh viên bổ sung</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Tổng thiết kế</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Newman assertions</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Pass Rate</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Bugs Found</t>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Bugs</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>FR-01 Register</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
-        <v>42</v>
-      </c>
-      <c r="C8" s="4" t="n">
+      <c r="B8" t="n">
+        <v>40</v>
+      </c>
+      <c r="C8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>46</v>
+      </c>
+      <c r="E8" t="n">
         <v>45</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="F8" t="n">
+        <v>45</v>
+      </c>
+      <c r="G8" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="n">
+      <c r="H8" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>FR-08 Checkout</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" t="n">
         <v>35</v>
       </c>
-      <c r="C9" s="4" t="n">
-        <v>136</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>34</v>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>80.0%</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="n">
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>40</v>
+      </c>
+      <c r="E9" t="n">
+        <v>76</v>
+      </c>
+      <c r="F9" t="n">
+        <v>76</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>FR-14 Category</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" t="n">
         <v>40</v>
       </c>
-      <c r="C10" s="4" t="n">
-        <v>36</v>
-      </c>
-      <c r="D10" s="4" t="n">
+      <c r="C10" t="n">
+        <v>7</v>
+      </c>
+      <c r="D10" t="n">
+        <v>47</v>
+      </c>
+      <c r="E10" t="n">
+        <v>112</v>
+      </c>
+      <c r="F10" t="n">
+        <v>112</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>90.0%</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>4</v>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
-        <v>117</v>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>217</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>85.1%</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="n">
+      <c r="B11" s="2" t="n">
+        <v>115</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>133</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>233</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>233</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2" t="n">
         <v>10</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>